<commit_message>
Expand curriculum to 22 tasks, fix Stage 1 alignments, correct 9 advanced blank templates, and implement database seeder upsert
</commit_message>
<xml_diff>
--- a/backend/media/templates/daily_showroom_footfall.xlsx
+++ b/backend/media/templates/daily_showroom_footfall.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -154,12 +154,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -528,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -674,49 +669,59 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Calculated Outputs:</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="C11" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E11" s="10" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Required calculations:</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>[B11] Total Weekly Walk-ins (SUM)</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>[C11] Avg Daily Yaris Drives (AVERAGE)</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>[D11] Avg Daily Corolla Drives (AVERAGE)</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>[E11] Total Days Recorded (COUNT)</t>
+    <row r="14">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>[B12] Total Weekly Walk-ins (SUM)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>[C12] Avg Daily Yaris Drives (AVERAGE)</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>[D12] Avg Daily Corolla Drives (AVERAGE)</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>[E12] Total Days Recorded (COUNT)</t>
         </is>
       </c>
     </row>

</xml_diff>